<commit_message>
Core V1 World Cup predictor with ML DC Monte Carlo odds and daily outputs
</commit_message>
<xml_diff>
--- a/outputs/daily/predictions_2026-06-12.xlsx
+++ b/outputs/daily/predictions_2026-06-12.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE3"/>
+  <dimension ref="A1:BL3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,225 +479,260 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>has_market</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>market_p_home</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>market_p_draw</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>market_p_away</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>market_p_over25</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>market_lambda_home</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>market_lambda_away</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>ml_p_home</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>ml_p_draw</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>ml_p_away</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>ml_p_over25</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>ml_p_btts_yes</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>dc_p_home</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>dc_p_draw</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>dc_p_away</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>dc_p_over25</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>dc_p_under25</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>dc_p_btts_yes</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>dc_p_btts_no</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>mc_p_home</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>mc_p_draw</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>mc_p_away</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>mc_p_over25</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>mc_p_btts_yes</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>mc_avg_home_goals</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>mc_avg_away_goals</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>mc_avg_total_goals</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>final_p_home</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>final_p_draw</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>final_p_away</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>pick</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>top_score_1</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>top_score_1_prob</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>top_score_2</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>top_score_2_prob</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>top_score_3</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>top_score_3_prob</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>top_score_4</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>top_score_4_prob</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>top_score_5</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>top_score_5_prob</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>top_score_6</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>top_score_6_prob</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>top_score_7</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>top_score_7_prob</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>top_score_8</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>top_score_8_prob</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>top_score_9</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>top_score_9_prob</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>top_score_10</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>top_score_10_prob</t>
         </is>
@@ -753,167 +788,188 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.888483195066821</v>
+        <v>1.729779118107939</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7344773283105702</v>
-      </c>
-      <c r="M2" t="n">
+        <v>0.8640531174118877</v>
+      </c>
+      <c r="M2" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.4972144846796657</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.2778551532033426</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.2249303621169916</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.4736842105263158</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1.599930327868852</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.9700696721311474</v>
+      </c>
+      <c r="T2" t="n">
         <v>0.5582819493341942</v>
       </c>
-      <c r="N2" t="n">
+      <c r="U2" t="n">
         <v>0.3324587766831252</v>
       </c>
-      <c r="O2" t="n">
+      <c r="V2" t="n">
         <v>0.1092592739826807</v>
       </c>
-      <c r="P2" t="n">
+      <c r="W2" t="n">
         <v>0.4624211232462194</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="X2" t="n">
         <v>0.3542608554359882</v>
       </c>
-      <c r="R2" t="n">
-        <v>0.6375792880390909</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.2341947551667954</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.1282259567941137</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0.4873166425818261</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.5126833574181739</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0.451598289361143</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0.548401710638857</v>
-      </c>
       <c r="Y2" t="n">
-        <v>0.6399049999999999</v>
+        <v>0.5676165731955537</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.23168</v>
+        <v>0.258126210821722</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.128415</v>
+        <v>0.1742572159827241</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.487495</v>
+        <v>0.4800198214219354</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.449815</v>
+        <v>0.5199801785780646</v>
       </c>
       <c r="AD2" t="n">
-        <v>1.889805</v>
+        <v>0.487128663272914</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.73197</v>
+        <v>0.512871336727086</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.621775</v>
+        <v>0.56853</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.5939657517513978</v>
+        <v>0.25636</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.2882399670007768</v>
+        <v>0.17511</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.1177942812478255</v>
-      </c>
-      <c r="AJ2" t="inlineStr">
+        <v>0.4803</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0.486245</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>1.730025</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0.8645</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>2.594525</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0.5361886194377227</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0.2920341858258614</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0.1717771947364159</v>
+      </c>
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>HOME</t>
         </is>
       </c>
-      <c r="AK2" t="n">
-        <v>0.5939657517513978</v>
-      </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AR2" t="n">
+        <v>0.5361886194377227</v>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="AT2" t="n">
+        <v>0.1228676873517065</v>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="AV2" t="n">
+        <v>0.1181022368576255</v>
+      </c>
+      <c r="AW2" t="inlineStr">
         <is>
           <t>2-0</t>
         </is>
       </c>
-      <c r="AM2" t="n">
-        <v>0.1294377917751458</v>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="AO2" t="n">
-        <v>0.1270129167576302</v>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="AQ2" t="n">
-        <v>0.1107513544278815</v>
-      </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AX2" t="n">
+        <v>0.111806026098679</v>
+      </c>
+      <c r="AY2" t="inlineStr">
         <is>
           <t>2-1</t>
         </is>
       </c>
-      <c r="AS2" t="n">
-        <v>0.09506912348542897</v>
-      </c>
-      <c r="AT2" t="inlineStr">
+      <c r="AZ2" t="n">
+        <v>0.09660634539599851</v>
+      </c>
+      <c r="BA2" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
       </c>
-      <c r="AU2" t="n">
-        <v>0.08265630682362626</v>
-      </c>
-      <c r="AV2" t="inlineStr">
+      <c r="BB2" t="n">
+        <v>0.08590304631414739</v>
+      </c>
+      <c r="BC2" t="inlineStr">
         <is>
           <t>3-0</t>
         </is>
       </c>
-      <c r="AW2" t="n">
-        <v>0.08148036485797373</v>
-      </c>
-      <c r="AX2" t="inlineStr">
+      <c r="BD2" t="n">
+        <v>0.06446657640804207</v>
+      </c>
+      <c r="BE2" t="inlineStr">
         <is>
           <t>3-1</t>
         </is>
       </c>
-      <c r="AY2" t="n">
-        <v>0.05984548069065503</v>
-      </c>
-      <c r="AZ2" t="inlineStr">
+      <c r="BF2" t="n">
+        <v>0.05570254631424041</v>
+      </c>
+      <c r="BG2" t="inlineStr">
         <is>
           <t>0-1</t>
         </is>
       </c>
-      <c r="BA2" t="n">
-        <v>0.04324593673703131</v>
-      </c>
-      <c r="BB2" t="inlineStr">
-        <is>
-          <t>4-0</t>
-        </is>
-      </c>
-      <c r="BC2" t="n">
-        <v>0.03846857494054914</v>
-      </c>
-      <c r="BD2" t="inlineStr">
+      <c r="BH2" t="n">
+        <v>0.05340371354135885</v>
+      </c>
+      <c r="BI2" t="inlineStr">
         <is>
           <t>1-2</t>
         </is>
       </c>
-      <c r="BE2" t="n">
-        <v>0.03697470859407612</v>
+      <c r="BJ2" t="n">
+        <v>0.0482564583115596</v>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="BL2" t="n">
+        <v>0.04173650695059104</v>
       </c>
     </row>
     <row r="3">
@@ -966,167 +1022,188 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1.630401482253932</v>
+        <v>1.710020340927313</v>
       </c>
       <c r="L3" t="n">
-        <v>1.004838341374228</v>
-      </c>
-      <c r="M3" t="n">
+        <v>0.944337579705359</v>
+      </c>
+      <c r="M3" t="b">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.5597905149839977</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.25720104742508</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.1830084375909223</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1.775163043478261</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.8948369565217392</v>
+      </c>
+      <c r="T3" t="n">
         <v>0.595624081293214</v>
       </c>
-      <c r="N3" t="n">
+      <c r="U3" t="n">
         <v>0.1883233378200571</v>
       </c>
-      <c r="O3" t="n">
+      <c r="V3" t="n">
         <v>0.2160525808867289</v>
       </c>
-      <c r="P3" t="n">
+      <c r="W3" t="n">
         <v>0.6060634664400587</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="X3" t="n">
         <v>0.494778992075029</v>
       </c>
-      <c r="R3" t="n">
-        <v>0.5080699055919224</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0.2704920055631597</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.2214380888449179</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.4903801548009806</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.5096198451990195</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.5214937181730891</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0.4785062818269109</v>
-      </c>
       <c r="Y3" t="n">
-        <v>0.509095</v>
+        <v>0.5426402346779358</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.268945</v>
+        <v>0.2616311868654818</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.22196</v>
+        <v>0.1957285784565826</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.490185</v>
+        <v>0.495128532813275</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.520335</v>
+        <v>0.504871467186725</v>
       </c>
       <c r="AD3" t="n">
-        <v>1.63134</v>
+        <v>0.5119039627265273</v>
       </c>
       <c r="AE3" t="n">
-        <v>1.00387</v>
+        <v>0.4880960372734727</v>
       </c>
       <c r="AF3" t="n">
-        <v>2.63521</v>
+        <v>0.544295</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.5562247022276328</v>
+        <v>0.259415</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.2252992383044533</v>
+        <v>0.19629</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.218476059467914</v>
-      </c>
-      <c r="AJ3" t="inlineStr">
+        <v>0.49521</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>0.5102</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>1.71074</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0.942885</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>2.653625</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>0.5680446931157079</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>0.2342013839234224</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>0.1977539229608697</v>
+      </c>
+      <c r="AQ3" t="inlineStr">
         <is>
           <t>HOME</t>
         </is>
       </c>
-      <c r="AK3" t="n">
-        <v>0.5562247022276328</v>
-      </c>
-      <c r="AL3" t="inlineStr">
+      <c r="AR3" t="n">
+        <v>0.5680446931157079</v>
+      </c>
+      <c r="AS3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
       </c>
-      <c r="AM3" t="n">
-        <v>0.1292152784964821</v>
-      </c>
-      <c r="AN3" t="inlineStr">
+      <c r="AT3" t="n">
+        <v>0.1249536872077475</v>
+      </c>
+      <c r="AU3" t="inlineStr">
         <is>
           <t>1-0</t>
         </is>
       </c>
-      <c r="AO3" t="n">
-        <v>0.1051559757499822</v>
-      </c>
-      <c r="AP3" t="inlineStr">
+      <c r="AV3" t="n">
+        <v>0.1089304612559015</v>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="AX3" t="n">
+        <v>0.1028490771015984</v>
+      </c>
+      <c r="AY3" t="inlineStr">
         <is>
           <t>2-1</t>
         </is>
       </c>
-      <c r="AQ3" t="n">
-        <v>0.09576035526841768</v>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="AS3" t="n">
-        <v>0.09529926489215648</v>
-      </c>
-      <c r="AT3" t="inlineStr">
+      <c r="AZ3" t="n">
+        <v>0.0971242485450533</v>
+      </c>
+      <c r="BA3" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
       </c>
-      <c r="AU3" t="n">
-        <v>0.08344870376053524</v>
-      </c>
-      <c r="AV3" t="inlineStr">
+      <c r="BB3" t="n">
+        <v>0.08170355271852653</v>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="BD3" t="n">
+        <v>0.05862467129644493</v>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="BF3" t="n">
+        <v>0.05536148020310704</v>
+      </c>
+      <c r="BG3" t="inlineStr">
         <is>
           <t>0-1</t>
         </is>
       </c>
-      <c r="AW3" t="n">
-        <v>0.06030193483828406</v>
-      </c>
-      <c r="AX3" t="inlineStr">
+      <c r="BH3" t="n">
+        <v>0.05506917615838143</v>
+      </c>
+      <c r="BI3" t="inlineStr">
         <is>
           <t>1-2</t>
         </is>
       </c>
-      <c r="AY3" t="n">
-        <v>0.05901839369300634</v>
-      </c>
-      <c r="AZ3" t="inlineStr">
-        <is>
-          <t>3-1</t>
-        </is>
-      </c>
-      <c r="BA3" t="n">
-        <v>0.05204260839026377</v>
-      </c>
-      <c r="BB3" t="inlineStr">
-        <is>
-          <t>3-0</t>
-        </is>
-      </c>
-      <c r="BC3" t="n">
-        <v>0.05179202091262734</v>
-      </c>
-      <c r="BD3" t="inlineStr">
+      <c r="BJ3" t="n">
+        <v>0.05363566479682946</v>
+      </c>
+      <c r="BK3" t="inlineStr">
         <is>
           <t>2-2</t>
         </is>
       </c>
-      <c r="BE3" t="n">
-        <v>0.04811183827866181</v>
+      <c r="BL3" t="n">
+        <v>0.0458590389008687</v>
       </c>
     </row>
   </sheetData>

</xml_diff>